<commit_message>
refactor: 消除 date/form 前缀，扁平化数据模型，拆分 src 为 reader/processing/render 三层
- 移除所有 date./form. 前缀：Sheet名直接作为context key，模板用 {{ Sheet名.字段 }}
- 移除旧格式兼容代码：reader 旧前缀检测、mapper _check_no_legacy_prefix
- mapper 新增 list 类型支持，YAML 列表数据不再被丢弃
- 拆分 src/ 目录：reader/ (xlsx+yaml+工厂函数) / processing/ (mapper+schema) / render/ (generator+filters)
- 同步更新 docs/ (用户指南/模板制作规范/开发手册) 和 tests/ (36/36 通过)
- .gitignore output/ 扩大到整个目录
</commit_message>
<xml_diff>
--- a/data/data_公司A.xlsx
+++ b/data/data_公司A.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="date.全局信息" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="date.基本情况" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全局信息" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="基本情况" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>